<commit_message>
RUN-2026-01 stage 6: extraction rules 0.3, second sample revision (725 items), simplified hand-coding and 70-row review sample
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/review/RUN-2026-01/G3_handcoding.xlsx
+++ b/review/RUN-2026-01/G3_handcoding.xlsx
@@ -8,15 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposed sample" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Passages" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hand-coded items" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Passages" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hand-coded items" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Instructions'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Proposed sample'!$A$1:$H$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Passages'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Hand-coded items'!$A$1:$O$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Instructions'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Passages'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hand-coded items'!$A$1:$F$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -460,7 +458,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Confirm or change the proposed sample (sheet 'Proposed sample').</t>
+          <t>Read a passage in sheet 'Passages'.</t>
         </is>
       </c>
     </row>
@@ -472,7 +470,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Read each passage (sheet 'Passages') and record every evidence item you find in sheet 'Hand-coded items', one row per item, before looking at any agent output.</t>
+          <t>In sheet 'Hand-coded items', add one row for each claim you find in it: pick its type, paste the sentence, and pick its scope.</t>
         </is>
       </c>
     </row>
@@ -484,7 +482,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>An item is one claim, of one information type, with its exact quote. If a sentence holds two claims of different types, use two rows.</t>
+          <t>Types: finding (judges the situation), recommendation (says what should happen), intervention (a law, strategy, system or programme), barrier (what blocks progress), outcome (result of a named action), lesson, metric (a number).</t>
         </is>
       </c>
     </row>
@@ -496,7 +494,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>information_type: finding, recommendation, intervention, barrier, outcome, lesson or metric (rules/extraction_rules.md section 2).</t>
+          <t>Scope: chapter (Chapter 2, workers), technology (the technology or digital issue itself is the subject), both, or out (not in scope).</t>
         </is>
       </c>
     </row>
@@ -508,7 +506,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>scope_basis: chapter, theme or both; themes: TECH codes from taxonomy/themes.csv, only where the passage materially concerns the area. Leave out incidental references.</t>
+          <t>If one sentence makes two claims of different types, use two rows with the same sentence. Leave the other columns empty.</t>
         </is>
       </c>
     </row>
@@ -520,470 +518,17 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Copy EU standard wording exactly into preparation_level or progress_level where it is used.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Leave a cell empty rather than guess. Add rows if needed.</t>
+          <t>Do this before looking at any agent output for these passages.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>family</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>language</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>reviewer_decision</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>reviewer_comment</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>MKD-EU-2020-001</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>EU</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>North Macedonia 2020 Report, SWD(2020) 351 final</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Chapter 2 section and summary; every section for technology and AI recommendations</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>EU: early Commission report (2020)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>MKD-EU-2023-001</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>EU</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>North Macedonia 2023 Report, SWD(2023) 693 final</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Chapter 2 section and summary; every section for technology and AI recommendations</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>EU: middle Commission report (2023)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>MKD-EU-2025-001</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>EU</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>North Macedonia 2025 Report, SWD(2025) 753 final</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Chapter 2 section and summary; every section for technology and AI recommendations</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>EU: latest Commission report (2025); includes hand-coding passages P1 and P2</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>MKD-EU-2025-003</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>EU</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Screening report North Macedonia, Cluster 2 - Internal Market</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Chapter 2 part in full; technology and AI material in the other Cluster 2 chapters</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>EU: other EU document (Cluster 2 screening report)</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>MKD-GOV-2021-001</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>GOV</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Закон за изменување и дополнување на законот за вработување и работа на странци (amending law), Official Gazette 163/21</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>mk</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>whole document</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>GOV: law amendment on employment of foreigners (Macedonian; tests machine translation)</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>MKD-GOV-2025-011</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>GOV</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Конечен извештај: Можност за употреба на вештачка интелигенција во јавниот сектор (State Audit Office performance audit: potential for use of AI in the public sector)</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>mk</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>summary, findings and recommendations</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>GOV: State Audit Office audit on AI in the public sector (Macedonian; implementation evidence for the theme)</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>MKD-IO-2024-001</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>North Macedonia Policy Notes</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>chapter 6 (Jobs and Migration) and chapter 11 (Digital Development)</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>IO: World Bank policy notes; includes hand-coding passage P3; 24 pages needed text recognition (difficult format)</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>MKD-IO-2021-001</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>How migration, human capital and the labour market interact in North Macedonia</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>findings on labour mobility, emigration and policy</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>IO: ETF report on migration and the labour market</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>MKD-RES-2023-001</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>RES</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Labor mobility preconditions for the regional economic integration: Pros and cons from Macedonian perspective (Policy Study No. 47)</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>findings and recommendations</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>RES: Finance Think study on labour mobility</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>MKD-CSO-2024-001</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>CSO</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Annual report on human rights in 2023</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>labour rights section</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>CSO: Helsinki Committee human rights report 2023</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>MKD-EU-2026-005</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>EU</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>EU-North Macedonia 21st Subcommittee on Innovation, Information Society and Social Policy</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>whole page</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Difficult format: webpage (EEAS readout of the 21st SA subcommittee, covering workers and digital transformation)</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H12"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1202,13 +747,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1217,15 +762,6 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="33" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1251,55 +787,10 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>speaker</t>
+          <t>scope</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>subjects</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>stated_status</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>preparation_level</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>progress_level</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>event_date</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>metric (indicator, value, unit)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>scope_basis</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>themes</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>flags</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1320,15 +811,6 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1345,15 +827,6 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1370,15 +843,6 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1395,15 +859,6 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
-      <c r="O5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1420,15 +875,6 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1445,15 +891,6 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1470,15 +907,6 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
-      <c r="O8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1495,15 +923,6 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1520,15 +939,6 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1545,15 +955,6 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="inlineStr"/>
-      <c r="O11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1570,15 +971,6 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1595,15 +987,6 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr"/>
-      <c r="O13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1620,15 +1003,6 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="inlineStr"/>
-      <c r="O14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1645,15 +1019,6 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="2" t="inlineStr"/>
-      <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1670,15 +1035,6 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr"/>
-      <c r="O16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1695,15 +1051,6 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="2" t="inlineStr"/>
-      <c r="O17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1720,15 +1067,6 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr"/>
-      <c r="O18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1745,15 +1083,6 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="inlineStr"/>
-      <c r="O19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1770,15 +1099,6 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="inlineStr"/>
-      <c r="O20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1795,15 +1115,6 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1820,15 +1131,6 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1845,15 +1147,6 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="2" t="inlineStr"/>
-      <c r="O23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1870,15 +1163,6 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1895,15 +1179,6 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="2" t="inlineStr"/>
-      <c r="O25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1920,15 +1195,6 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1945,15 +1211,6 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1970,15 +1227,6 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1995,15 +1243,6 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr"/>
-      <c r="N29" s="2" t="inlineStr"/>
-      <c r="O29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2020,15 +1259,6 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr"/>
-      <c r="O30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2045,15 +1275,6 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
-      <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
-      <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="2" t="inlineStr"/>
-      <c r="O31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2070,15 +1291,6 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
-      <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr"/>
-      <c r="O32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2095,15 +1307,6 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr"/>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr"/>
-      <c r="O33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2120,15 +1323,6 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr"/>
-      <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
-      <c r="O34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2145,15 +1339,6 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr"/>
-      <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="2" t="inlineStr"/>
-      <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr"/>
-      <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="2" t="inlineStr"/>
-      <c r="O35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2170,15 +1355,6 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr"/>
-      <c r="O36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2195,18 +1371,17 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
-      <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr"/>
-      <c r="M37" s="2" t="inlineStr"/>
-      <c r="N37" s="2" t="inlineStr"/>
-      <c r="O37" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O37"/>
+  <autoFilter ref="A1:F37"/>
+  <dataValidations count="2">
+    <dataValidation sqref="C2:C37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"finding,recommendation,intervention,barrier,outcome,lesson,metric"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"chapter,technology,both,out"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
RUN-2026-01 stage 6: independent G3 review (blind coding, 725 items checked), routine fixes, sample now 775 items
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/review/RUN-2026-01/G3_handcoding.xlsx
+++ b/review/RUN-2026-01/G3_handcoding.xlsx
@@ -807,10 +807,26 @@
           <t>1</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>North Macedonia is at an early stage of preparation  on the freedom of movement for workers, and no progress was made in this area.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>chapter</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12).</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -823,10 +839,26 @@
           <t>2</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>The Commission’s recommendations from last year were not implemented and therefore remain valid.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>chapter</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Implementation status of earlier recommendations; treated as a finding, not a lead-in, because it makes its own claim.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -839,10 +871,26 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>strengthen the capacity of the Employment Service Agency, by continuing to organise training, and further align legislation and the exchange of good practices, in line with the European Employment Services (EURES) and European Labour Authority (ELA) regulations;</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>chapter</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -855,10 +903,26 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>continue to align  the legal framework to the EU acquis on access to the labour market, particularly to rules on non -discrimination on grounds of nationality against EU workers in all sectors;</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>chapter</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -871,10 +935,26 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>continue to negotiate and conclude bilateral agreements on social security coordination and healthcare insurance with EU Member States</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>chapter</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Bullet split into two claims: bilateral agreements (chapter only) and administrative measures for electronic exchange (chapter and technology).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -887,106 +967,218 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>put in place administrative measures to prepare for accession and for electronic exchange of social security data.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Electronic exchange of social security data with the EU (EESSI-type interoperability) meets the materiality test (TECH-INTEROP); 'prepare for accession' part alone would be chapter only.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>The country is moderately prepared in the area of digital transformation and media.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Chapter 10 is not an in-scope chapter; the claim covers digital transformation and media together, so only partly technology (TECH-DIGI); theme_doubtful.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Some  progress was made  to harmonise  the legal framework with the EU acquis  as part of the Reform Agenda commitments , by adopting a cybersecurity strategy and with a slight increase in electronic services available to citizens and businesses.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Progress judgement (TECH-CYBER, TECH-DGOV); the adoption of the strategy is a separate intervention row.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>intervention</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>by adopting a cybersecurity strategy</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Intervention clause split from the progress finding in the same sentence (TECH-CYBER).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>The Commission’s recommendations from last year were only partially implemented and therefore remain largely valid.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Refers to last year's Chapter 10 recommendations, which mix digital and media; theme_doubtful.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Continue aligning with the European Electronic Communications Code, the EU Gigabit Infrastructure Act (GIA) the EU Directive on security of network and information systems (the NIS2 Directive) and the 5G cybersecurity toolbox;</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). TECH-INFRA and TECH-CYBER.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>increase efforts to strengthen the independence and capacity of the media regulator, the public service broadcaster and the regulator on electronic communication;</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Difficult: only the electronic communications regulator part arguably meets the test (TECH-INFRA); media regulator and public broadcaster are out. Kept as one item because the verb is shared; theme_doubtful.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -996,189 +1188,381 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>continue to improve the 112 emergency number service by ensuring sufficient human resources.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>out</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). 112 staffing is out of scope under section 4 and the TECH-INFRA incidental example.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Investing in digital development, aligned with the EU Digital Agenda 2030, presents a strategic opportunity for North Macedonia to foster sustainable growth and resilience.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Judgement about opportunity rather than current state; closest type is finding (TECH-DIGI); ambiguous_type.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>With a relatively high internet usage rate and widespread access to digital devices among its citizens, the country is poised to stimulate job creation and enhance economic competitiveness.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Forward-looking assessment; closest to finding (TECH-DIGI, TECH-INFRA).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>To fully capitalize on digitalization and harness the potential of technologies like artificial intelligence, cloud computing, and big data, North Macedonia should prioritize the development of modern data hosting infrastructure, ensure affordable digital services for all, and promote digital skills among its people and businesses.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Digital skills kept inside this item because the same sentence ties them to AI and digitalisation; not extracted separately.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Given its small economy, North Macedonia could accelerate digitalization through a regional approach within the Western Balkans, focusing on investments in regional digital infrastructure, such as fiber-optic links and large data centers, as well as harmonized telecommunications (telecoms) and cybersecurity policies.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Line-break hyphen in 'fiber-optic' joined; check quote against converted text.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Over four-fifths (83 percent) of North Macedonia’s population used the internet in 2021,41 on par with regional averages, but with a pronounced gender gap.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Footnote marker 41 left in quote as printed. Internet usage treated as material (digital adoption is the subject), though close to the TECH-INFRA incidental example.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>North Macedonia’s internet usage rates place it ahead of 10 of 19 countries in the ECA region.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>While the rural/ urban divide is negligible, with a gap of only 0.7 percentage points in internet use,42 internet access is lower among women, at 79.2 percent, compared to 83.5 percent among men.43</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Line break inside 'rural/urban' reproduced as a space by the converter join; footnote markers left in.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>The quality of fixed internet access is quite high compared to EU countries, but prices remain unaffordable for the poorest.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). TECH-INFRA.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Internet speed in North Macedonia is relatively high for fixed broadband, at 48 megabits per second (Mbps) in 2023, slightly above the ECA average but about 53 Mbps slower than in high-income countries.</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Mobile broadband speeds are on par with the regional average.44</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Comparative statement with no number; finding rather than metric (ambiguous_type).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Affordability is a greater challenge, however,</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Sentence split: qualitative judgement (finding) and the price figures (metric).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1188,13 +1572,29 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>as fixed broadband prices45 are well above the affordability threshold of 2 percent of gross national income46 set by the Broadband Commission as a threshold for affordability, and mobile broadband prices are at around 1 percent.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1204,13 +1604,29 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>barrier</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>These high costs maintain a digital divide and restrict the inclusiveness of digital services within the population.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Explains what restricts digital inclusion; barrier rather than finding.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1220,13 +1636,29 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr"/>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Increasing competition on both retail and wholesale telecoms markets would help reduce this key barrier to adoption.</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Phrased conditionally ('would help') but forward-looking; recommendation.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1236,141 +1668,93 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr"/>
-      <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr"/>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>finding</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>North Macedonia’s data hosting capacity does not compare well with peers</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Coded blind by an independent agent (decision E12). Sentence is cut off at the end of the passage ('and demand' continues on the next page); quote limited to the complete clause.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr"/>
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr"/>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="2" t="inlineStr"/>
-      <c r="F31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr"/>
-      <c r="D33" s="2" t="inlineStr"/>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr"/>
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr"/>
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="2" t="inlineStr"/>
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr"/>
-      <c r="D37" s="2" t="inlineStr"/>
-      <c r="E37" s="2" t="inlineStr"/>
-      <c r="F37" s="2" t="inlineStr"/>
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F37"/>

</xml_diff>